<commit_message>
Multiple rules to sheet
</commit_message>
<xml_diff>
--- a/data/aggreg.xlsx
+++ b/data/aggreg.xlsx
@@ -41,7 +41,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -52,6 +52,12 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -83,18 +89,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -405,129 +408,129 @@
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="5" width="5.576428571428571" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="5" width="6.147857142857143" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="5" width="6.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="5" width="5.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="5" width="5.576428571428571" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="4" width="5.576428571428571" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="4" width="6.147857142857143" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="4" width="6.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="4" width="5.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="4" width="5.576428571428571" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="4" t="s">
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="2">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
+      <c r="A2" s="3">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3">
+        <v>1</v>
+      </c>
+      <c r="C2" s="3">
         <v>3</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="3">
         <v>5</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="3">
         <v>10</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="2">
-        <v>1</v>
-      </c>
-      <c r="B3" s="2">
-        <v>1</v>
-      </c>
-      <c r="C3" s="2">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
+      <c r="A3" s="3">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3">
+        <v>1</v>
+      </c>
+      <c r="C3" s="3">
         <v>6</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="3">
         <v>6</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="3">
         <v>20</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="2">
-        <v>1</v>
-      </c>
-      <c r="B4" s="2">
-        <v>1</v>
-      </c>
-      <c r="C4" s="2">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
+      <c r="A4" s="3">
+        <v>1</v>
+      </c>
+      <c r="B4" s="3">
+        <v>1</v>
+      </c>
+      <c r="C4" s="3">
         <v>9</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="3">
         <v>7</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="3">
         <v>30</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="2">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
+      <c r="A5" s="3">
         <v>2</v>
       </c>
-      <c r="B5" s="2">
-        <v>1</v>
-      </c>
-      <c r="C5" s="2">
+      <c r="B5" s="3">
+        <v>1</v>
+      </c>
+      <c r="C5" s="3">
         <v>9</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="3">
         <v>7</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="3">
         <v>20</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="2">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
+      <c r="A6" s="3">
         <v>3</v>
       </c>
-      <c r="B6" s="2">
-        <v>1</v>
-      </c>
-      <c r="C6" s="2">
+      <c r="B6" s="3">
+        <v>1</v>
+      </c>
+      <c r="C6" s="3">
         <v>9</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="3">
         <v>7</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="3">
         <v>20</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="2">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
+      <c r="A7" s="3">
         <v>4</v>
       </c>
-      <c r="B7" s="2">
-        <v>1</v>
-      </c>
-      <c r="C7" s="2">
+      <c r="B7" s="3">
+        <v>1</v>
+      </c>
+      <c r="C7" s="3">
         <v>9</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="3">
         <v>7</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="3">
         <v>20</v>
       </c>
     </row>
@@ -544,11 +547,11 @@
   <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="3" width="5.576428571428571" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="3" width="6.147857142857143" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="3" width="6.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="3" width="5.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="3" width="5.576428571428571" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="4" width="5.576428571428571" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="4" width="6.147857142857143" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="4" width="6.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="4" width="5.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="4" width="5.576428571428571" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -569,70 +572,70 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="1">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2">
         <v>3</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2" s="2">
         <v>9</v>
       </c>
-      <c r="D2" s="1">
+      <c r="D2" s="2">
         <v>5</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>20</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" s="2">
-        <v>1</v>
-      </c>
-      <c r="C3" s="2">
+      <c r="B3" s="3">
+        <v>1</v>
+      </c>
+      <c r="C3" s="3">
         <v>9</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="3">
         <v>7</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="3">
         <v>20</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="2">
+      <c r="A4" s="3">
         <v>3</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4" s="2">
         <v>0</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="2">
         <v>0</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="2">
         <v>0</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>5</v>
       </c>
-      <c r="B5" s="1">
-        <v>1</v>
-      </c>
-      <c r="C5" s="2">
+      <c r="B5" s="2">
+        <v>1</v>
+      </c>
+      <c r="C5" s="3">
         <v>9</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="3">
         <v>7</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="3">
         <v>20</v>
       </c>
     </row>

</xml_diff>